<commit_message>
chore: resolve binary conflict on IP formatting template
Source/Data/IpAddressConditionalFormattingTemplate.xlsx changed on this branch
only via the build refresh in 865f59a (no deliberate template edit), and develop
re-saved it the same way. Reset to develop copy to clear the merge conflict. The
PreBuild step reapplies the conditional-formatting rules on build.
</commit_message>
<xml_diff>
--- a/Source/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Source/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="325">
+  <dxfs count="350">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,181 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -2964,31 +3139,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="320">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="345">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="321">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="346">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="322">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="347">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="322">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="347">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="322">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="347">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="323">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="348">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="323">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="348">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="323">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="348">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="324">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="349">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
chore(data): update IP address conditional formatting template
</commit_message>
<xml_diff>
--- a/Source/Data/IpAddressConditionalFormattingTemplate.xlsx
+++ b/Source/Data/IpAddressConditionalFormattingTemplate.xlsx
@@ -195,7 +195,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="360">
+  <dxfs count="375">
     <dxf>
       <fill>
         <patternFill>
@@ -262,6 +262,111 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffadd8e6"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ff59abf8"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="ffffb6c1"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fffacd90"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
+    <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <fill>
+        <patternFill>
+          <bgColor rgb="fff2ceef"/>
+        </patternFill>
+      </fill>
+    </d:dxf>
     <d:dxf xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <fill>
         <patternFill>
@@ -3209,31 +3314,31 @@
     <row r="78" ht="15" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A:A">
-    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="355">
+    <cfRule priority="1" type="containsText" operator="containsText" text="microsoft" stopIfTrue="1" dxfId="370">
       <formula>NOT(ISERROR(SEARCH("microsoft",A1)))</formula>
     </cfRule>
-    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="356">
+    <cfRule priority="2" type="containsText" operator="containsText" text="proofpoint" stopIfTrue="1" dxfId="371">
       <formula>NOT(ISERROR(SEARCH("proofpoint",A1)))</formula>
     </cfRule>
-    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="357">
+    <cfRule priority="3" type="containsText" operator="containsText" text=" vpn" stopIfTrue="1" dxfId="372">
       <formula>NOT(ISERROR(SEARCH(" vpn",A1)))</formula>
     </cfRule>
-    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="357">
+    <cfRule priority="4" type="containsText" operator="containsText" text=" tor" stopIfTrue="1" dxfId="372">
       <formula>NOT(ISERROR(SEARCH(" tor",A1)))</formula>
     </cfRule>
-    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="357">
+    <cfRule priority="5" type="containsText" operator="containsText" text=" proxy" stopIfTrue="1" dxfId="372">
       <formula>NOT(ISERROR(SEARCH(" proxy",A1)))</formula>
     </cfRule>
-    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="358">
+    <cfRule priority="6" type="containsText" operator="containsText" text=" hosting" stopIfTrue="1" dxfId="373">
       <formula>NOT(ISERROR(SEARCH(" hosting",A1)))</formula>
     </cfRule>
-    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="358">
+    <cfRule priority="7" type="containsText" operator="containsText" text=" cloud" stopIfTrue="1" dxfId="373">
       <formula>NOT(ISERROR(SEARCH(" cloud",A1)))</formula>
     </cfRule>
-    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="358">
+    <cfRule priority="8" type="containsText" operator="containsText" text=" datacenter" stopIfTrue="1" dxfId="373">
       <formula>NOT(ISERROR(SEARCH(" datacenter",A1)))</formula>
     </cfRule>
-    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="359">
+    <cfRule priority="9" type="containsText" operator="containsText" text="mobile" stopIfTrue="1" dxfId="374">
       <formula>NOT(ISERROR(SEARCH("mobile",A1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>